<commit_message>
Fix workbook rejected by Excel: one cached value per formula cell
openpyxl already writes an empty <v/> placeholder after each <f>, so
appending the computed value produced two <v> elements in the same cell.
A cell may carry only one, and Excel refuses to open the file. The
injection now replaces the placeholder instead of adding to it.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Up6mzUYyYRDCaMaWzFtptk
</commit_message>
<xml_diff>
--- a/receipts/Receipt_Details_Sejal_Ria.xlsx
+++ b/receipts/Receipt_Details_Sejal_Ria.xlsx
@@ -672,7 +672,6 @@
       <c r="I5" s="9">
         <f>SUM(F5:H5)</f>
         <v>0</v>
-        <v/>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
@@ -715,7 +714,6 @@
       <c r="I6" s="9">
         <f>SUM(F6:H6)</f>
         <v>5100</v>
-        <v/>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
@@ -758,7 +756,6 @@
       <c r="I7" s="9">
         <f>SUM(F7:H7)</f>
         <v>500</v>
-        <v/>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
@@ -801,7 +798,6 @@
       <c r="I8" s="9">
         <f>SUM(F8:H8)</f>
         <v>1000</v>
-        <v/>
       </c>
       <c r="J8" s="10" t="inlineStr">
         <is>
@@ -844,7 +840,6 @@
       <c r="I9" s="9">
         <f>SUM(F9:H9)</f>
         <v>501</v>
-        <v/>
       </c>
       <c r="J9" s="10" t="inlineStr">
         <is>
@@ -883,7 +878,6 @@
       <c r="I10" s="9">
         <f>SUM(F10:H10)</f>
         <v>501</v>
-        <v/>
       </c>
       <c r="J10" s="10" t="inlineStr">
         <is>
@@ -922,7 +916,6 @@
       <c r="I11" s="9">
         <f>SUM(F11:H11)</f>
         <v>1100</v>
-        <v/>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
@@ -965,7 +958,6 @@
       <c r="I12" s="9">
         <f>SUM(F12:H12)</f>
         <v>1100</v>
-        <v/>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
@@ -1004,7 +996,6 @@
       <c r="I13" s="9">
         <f>SUM(F13:H13)</f>
         <v>500</v>
-        <v/>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
@@ -1043,7 +1034,6 @@
       <c r="I14" s="9">
         <f>SUM(F14:H14)</f>
         <v>500</v>
-        <v/>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
@@ -1082,7 +1072,6 @@
       <c r="I15" s="9">
         <f>SUM(F15:H15)</f>
         <v>1100</v>
-        <v/>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
@@ -1121,7 +1110,6 @@
       <c r="I16" s="9">
         <f>SUM(F16:H16)</f>
         <v>1100</v>
-        <v/>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
@@ -1160,7 +1148,6 @@
       <c r="I17" s="9">
         <f>SUM(F17:H17)</f>
         <v>1100</v>
-        <v/>
       </c>
       <c r="J17" s="10" t="inlineStr">
         <is>
@@ -1203,7 +1190,6 @@
       <c r="I18" s="9">
         <f>SUM(F18:H18)</f>
         <v>1100</v>
-        <v/>
       </c>
       <c r="J18" s="10" t="inlineStr">
         <is>
@@ -1244,7 +1230,6 @@
       <c r="I19" s="9">
         <f>SUM(F19:H19)</f>
         <v>1000</v>
-        <v/>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
@@ -1287,7 +1272,6 @@
       <c r="I20" s="9">
         <f>SUM(F20:H20)</f>
         <v>500</v>
-        <v/>
       </c>
       <c r="J20" s="10" t="inlineStr">
         <is>
@@ -1330,7 +1314,6 @@
       <c r="I21" s="9">
         <f>SUM(F21:H21)</f>
         <v>500</v>
-        <v/>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
@@ -1369,7 +1352,6 @@
       <c r="I22" s="9">
         <f>SUM(F22:H22)</f>
         <v>500</v>
-        <v/>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
@@ -1408,7 +1390,6 @@
       <c r="I23" s="9">
         <f>SUM(F23:H23)</f>
         <v>500</v>
-        <v/>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
@@ -1447,7 +1428,6 @@
       <c r="I24" s="9">
         <f>SUM(F24:H24)</f>
         <v>500</v>
-        <v/>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
@@ -1486,7 +1466,6 @@
       <c r="I25" s="9">
         <f>SUM(F25:H25)</f>
         <v>1100</v>
-        <v/>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
@@ -1525,7 +1504,6 @@
       <c r="I26" s="9">
         <f>SUM(F26:H26)</f>
         <v>1100</v>
-        <v/>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
@@ -1564,7 +1542,6 @@
       <c r="I27" s="9">
         <f>SUM(F27:H27)</f>
         <v>701</v>
-        <v/>
       </c>
       <c r="J27" s="10" t="inlineStr">
         <is>
@@ -1603,7 +1580,6 @@
       <c r="I28" s="9">
         <f>SUM(F28:H28)</f>
         <v>700</v>
-        <v/>
       </c>
       <c r="J28" s="10" t="inlineStr">
         <is>
@@ -1642,7 +1618,6 @@
       <c r="I29" s="9">
         <f>SUM(F29:H29)</f>
         <v>500</v>
-        <v/>
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
@@ -1681,7 +1656,6 @@
       <c r="I30" s="9">
         <f>SUM(F30:H30)</f>
         <v>500</v>
-        <v/>
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
@@ -1720,7 +1694,6 @@
       <c r="I31" s="9">
         <f>SUM(F31:H31)</f>
         <v>500</v>
-        <v/>
       </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
@@ -1759,7 +1732,6 @@
       <c r="I32" s="9">
         <f>SUM(F32:H32)</f>
         <v>500</v>
-        <v/>
       </c>
       <c r="J32" s="10" t="inlineStr">
         <is>
@@ -1798,7 +1770,6 @@
       <c r="I33" s="9">
         <f>SUM(F33:H33)</f>
         <v>500</v>
-        <v/>
       </c>
       <c r="J33" s="10" t="inlineStr">
         <is>
@@ -1837,7 +1808,6 @@
       <c r="I34" s="9">
         <f>SUM(F34:H34)</f>
         <v>500</v>
-        <v/>
       </c>
       <c r="J34" s="10" t="inlineStr">
         <is>
@@ -1876,7 +1846,6 @@
       <c r="I35" s="9">
         <f>SUM(F35:H35)</f>
         <v>500</v>
-        <v/>
       </c>
       <c r="J35" s="10" t="inlineStr">
         <is>
@@ -1915,7 +1884,6 @@
       <c r="I36" s="9">
         <f>SUM(F36:H36)</f>
         <v>501</v>
-        <v/>
       </c>
       <c r="J36" s="4" t="inlineStr">
         <is>
@@ -1954,7 +1922,6 @@
       <c r="I37" s="9">
         <f>SUM(F37:H37)</f>
         <v>501</v>
-        <v/>
       </c>
       <c r="J37" s="4" t="inlineStr">
         <is>
@@ -1993,7 +1960,6 @@
       <c r="I38" s="9">
         <f>SUM(F38:H38)</f>
         <v>500</v>
-        <v/>
       </c>
       <c r="J38" s="10" t="inlineStr">
         <is>
@@ -2032,7 +1998,6 @@
       <c r="I39" s="9">
         <f>SUM(F39:H39)</f>
         <v>500</v>
-        <v/>
       </c>
       <c r="J39" s="10" t="inlineStr">
         <is>
@@ -2071,7 +2036,6 @@
       <c r="I40" s="9">
         <f>SUM(F40:H40)</f>
         <v>500</v>
-        <v/>
       </c>
       <c r="J40" s="4" t="inlineStr">
         <is>
@@ -2110,7 +2074,6 @@
       <c r="I41" s="9">
         <f>SUM(F41:H41)</f>
         <v>1001</v>
-        <v/>
       </c>
       <c r="J41" s="10" t="inlineStr">
         <is>
@@ -2149,7 +2112,6 @@
       <c r="I42" s="9">
         <f>SUM(F42:H42)</f>
         <v>501</v>
-        <v/>
       </c>
       <c r="J42" s="4" t="inlineStr">
         <is>
@@ -2192,7 +2154,6 @@
       <c r="I43" s="9">
         <f>SUM(F43:H43)</f>
         <v>501</v>
-        <v/>
       </c>
       <c r="J43" s="4" t="inlineStr">
         <is>
@@ -2235,7 +2196,6 @@
       <c r="I44" s="9">
         <f>SUM(F44:H44)</f>
         <v>501</v>
-        <v/>
       </c>
       <c r="J44" s="10" t="inlineStr">
         <is>
@@ -2278,7 +2238,6 @@
       <c r="I45" s="9">
         <f>SUM(F45:H45)</f>
         <v>500</v>
-        <v/>
       </c>
       <c r="J45" s="10" t="inlineStr">
         <is>
@@ -2317,7 +2276,6 @@
       <c r="I46" s="9">
         <f>SUM(F46:H46)</f>
         <v>501</v>
-        <v/>
       </c>
       <c r="J46" s="10" t="inlineStr">
         <is>
@@ -2356,7 +2314,6 @@
       <c r="I47" s="9">
         <f>SUM(F47:H47)</f>
         <v>1251</v>
-        <v/>
       </c>
       <c r="J47" s="10" t="inlineStr">
         <is>
@@ -2399,7 +2356,6 @@
       <c r="I48" s="9">
         <f>SUM(F48:H48)</f>
         <v>751</v>
-        <v/>
       </c>
       <c r="J48" s="10" t="inlineStr">
         <is>
@@ -2442,7 +2398,6 @@
       <c r="I49" s="9">
         <f>SUM(F49:H49)</f>
         <v>1001</v>
-        <v/>
       </c>
       <c r="J49" s="10" t="inlineStr">
         <is>
@@ -2481,7 +2436,6 @@
       <c r="I50" s="9">
         <f>SUM(F50:H50)</f>
         <v>1000</v>
-        <v/>
       </c>
       <c r="J50" s="10" t="inlineStr">
         <is>
@@ -2520,7 +2474,6 @@
       <c r="I51" s="9">
         <f>SUM(F51:H51)</f>
         <v>500</v>
-        <v/>
       </c>
       <c r="J51" s="10" t="inlineStr">
         <is>
@@ -2563,7 +2516,6 @@
       <c r="I52" s="9">
         <f>SUM(F52:H52)</f>
         <v>501</v>
-        <v/>
       </c>
       <c r="J52" s="10" t="inlineStr">
         <is>
@@ -2602,7 +2554,6 @@
       <c r="I53" s="9">
         <f>SUM(F53:H53)</f>
         <v>2500</v>
-        <v/>
       </c>
       <c r="J53" s="10" t="inlineStr">
         <is>
@@ -2645,7 +2596,6 @@
       <c r="I54" s="9">
         <f>SUM(F54:H54)</f>
         <v>2500</v>
-        <v/>
       </c>
       <c r="J54" s="10" t="inlineStr">
         <is>
@@ -2688,7 +2638,6 @@
       <c r="I55" s="9">
         <f>SUM(F55:H55)</f>
         <v>1101</v>
-        <v/>
       </c>
       <c r="J55" s="10" t="inlineStr">
         <is>
@@ -2731,7 +2680,6 @@
       <c r="I56" s="9">
         <f>SUM(F56:H56)</f>
         <v>1101</v>
-        <v/>
       </c>
       <c r="J56" s="10" t="inlineStr">
         <is>
@@ -2774,7 +2722,6 @@
       <c r="I57" s="9">
         <f>SUM(F57:H57)</f>
         <v>701</v>
-        <v/>
       </c>
       <c r="J57" s="10" t="inlineStr">
         <is>
@@ -2817,7 +2764,6 @@
       <c r="I58" s="9">
         <f>SUM(F58:H58)</f>
         <v>701</v>
-        <v/>
       </c>
       <c r="J58" s="10" t="inlineStr">
         <is>
@@ -2860,7 +2806,6 @@
       <c r="I59" s="9">
         <f>SUM(F59:H59)</f>
         <v>200</v>
-        <v/>
       </c>
       <c r="J59" s="10" t="inlineStr">
         <is>
@@ -2903,7 +2848,6 @@
       <c r="I60" s="9">
         <f>SUM(F60:H60)</f>
         <v>300</v>
-        <v/>
       </c>
       <c r="J60" s="10" t="inlineStr">
         <is>
@@ -2946,7 +2890,6 @@
       <c r="I61" s="9">
         <f>SUM(F61:H61)</f>
         <v>500</v>
-        <v/>
       </c>
       <c r="J61" s="10" t="inlineStr">
         <is>
@@ -2985,7 +2928,6 @@
       <c r="I62" s="9">
         <f>SUM(F62:H62)</f>
         <v>500</v>
-        <v/>
       </c>
       <c r="J62" s="10" t="inlineStr">
         <is>
@@ -3022,7 +2964,6 @@
       <c r="I63" s="9">
         <f>SUM(F63:H63)</f>
         <v>15000</v>
-        <v/>
       </c>
       <c r="J63" s="10" t="inlineStr">
         <is>
@@ -3048,22 +2989,18 @@
       <c r="F64" s="12">
         <f>SUM(F5:F63)</f>
         <v>13453</v>
-        <v/>
       </c>
       <c r="G64" s="12">
         <f>SUM(G5:G63)</f>
         <v>16804</v>
-        <v/>
       </c>
       <c r="H64" s="12">
         <f>SUM(H5:H63)</f>
         <v>31661</v>
-        <v/>
       </c>
       <c r="I64" s="12">
         <f>SUM(I5:I63)</f>
         <v>61918</v>
-        <v/>
       </c>
       <c r="J64" s="11" t="n"/>
       <c r="K64" s="11" t="n"/>
@@ -3141,12 +3078,10 @@
       <c r="B5" s="6">
         <f>SUM('Receipt Details'!F5:F63)</f>
         <v>13453</v>
-        <v/>
       </c>
       <c r="C5" s="16">
         <f>COUNT('Receipt Details'!F5:F63)</f>
         <v>16</v>
-        <v/>
       </c>
     </row>
     <row r="6">
@@ -3158,12 +3093,10 @@
       <c r="B6" s="7">
         <f>SUM('Receipt Details'!G5:G63)</f>
         <v>16804</v>
-        <v/>
       </c>
       <c r="C6" s="16">
         <f>COUNT('Receipt Details'!G5:G63)</f>
         <v>14</v>
-        <v/>
       </c>
     </row>
     <row r="7">
@@ -3175,12 +3108,10 @@
       <c r="B7" s="8">
         <f>SUM('Receipt Details'!H5:H63)</f>
         <v>31661</v>
-        <v/>
       </c>
       <c r="C7" s="16">
         <f>COUNT('Receipt Details'!H5:H63)</f>
         <v>29</v>
-        <v/>
       </c>
     </row>
     <row r="8">
@@ -3192,12 +3123,10 @@
       <c r="B8" s="18">
         <f>SUM(B5:B7)</f>
         <v>61918</v>
-        <v/>
       </c>
       <c r="C8" s="19">
         <f>SUM(C5:C7)</f>
         <v>59</v>
-        <v/>
       </c>
     </row>
     <row r="10">
@@ -3216,7 +3145,6 @@
       <c r="B11" s="21">
         <f>B5+B7/2</f>
         <v>29283.5</v>
-        <v/>
       </c>
     </row>
     <row r="12">
@@ -3228,7 +3156,6 @@
       <c r="B12" s="22">
         <f>B6+B7/2</f>
         <v>32634.5</v>
-        <v/>
       </c>
     </row>
     <row r="14">
@@ -3247,7 +3174,6 @@
       <c r="B15" s="23">
         <f>SUMIF('Receipt Details'!E5:E63,1,'Receipt Details'!I5:I63)</f>
         <v>24303</v>
-        <v/>
       </c>
     </row>
     <row r="16">
@@ -3269,7 +3195,6 @@
       <c r="B17" s="24">
         <f>B15-B16</f>
         <v>0</v>
-        <v/>
       </c>
     </row>
     <row r="18">
@@ -3281,7 +3206,6 @@
       <c r="B18" s="23">
         <f>B8</f>
         <v>61918</v>
-        <v/>
       </c>
     </row>
     <row r="19">
@@ -3303,7 +3227,6 @@
       <c r="B20" s="24">
         <f>B18-B19</f>
         <v>-67</v>
-        <v/>
       </c>
     </row>
     <row r="22">

</xml_diff>